<commit_message>
Add walk with walking song, Help Mommy cooking module, drop photos
From the 1 Oct standup:
- Rename Skattejakt to Letejakt (Search hunt)
- New Gå på tur module: tick off things seen on a walk, then Monki plays a
  walking song built from the child's picks (concept for an AI jingle)
- New Hjelp mamma module: 10 example Norwegian family dishes with
  child-sized jobs and a safety note for the grown-up
- Remove all photo prompts to avoid collecting images of children; the
  month-24 reward is now a printed poster instead of a photo card
- Hub regrouped: Play (hunt, walk), Feelings, Together (food, songs)
- 14 new voice lines; voice script sheet regenerated (57 lines)
- deck-screenshots/no: 22 phone screenshots for the pitch deck

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011jBTVcGqAJdvug1cHrdZNw
</commit_message>
<xml_diff>
--- a/voice/voice-script.xlsx
+++ b/voice/voice-script.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How to record" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Script'!$A$1:$J$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Script'!$A$1:$J$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1658,12 +1658,12 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Skattejakt! Gå ut sammen og finn noe rødt, noe mykt, noe rundt og et blad. Trykk når du har funnet det!</t>
+          <t>Letejakt! Gå ut sammen og finn noe rødt, noe mykt, noe rundt og et blad. Trykk når du har funnet det!</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Treasure hunt! Go outside together and find something red, something soft, something round and a leaf. Tap when you find it!</t>
+          <t>Search hunt! Go outside together and find something red, something soft, something round and a leaf. Tap when you find it!</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2201,47 +2201,607 @@
       <c r="J43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="n">
+      <c r="A44" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="3" t="inlineStr"/>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>Monki</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Go for a walk</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>walkSay.mp3</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Nå går vi på tur! Trykk på alt du ser underveis.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Let's go for a walk! Tap everything you see on the way.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Outdoorsy, excited to go</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Go for a walk</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>walkItems-bird.mp3</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Fugl</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Bird</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Naming it happily, one word</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Go for a walk</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>walkItems-dog.mp3</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Hund</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Dog</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Naming it happily, one word</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Go for a walk</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>walkItems-tree.mp3</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Tre</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Tree</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Naming it happily, one word</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr"/>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Go for a walk</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>walkItems-flower.mp3</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Blomst</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Flower</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Naming it happily, one word</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr"/>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Go for a walk</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>walkItems-bus.mp3</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Buss</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Bus</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Naming it happily, one word</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr"/>
+      <c r="J49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr"/>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Go for a walk</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>walkItems-cat.mp3</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Katt</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Cat</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Naming it happily, one word</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr"/>
+      <c r="J50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr"/>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Go for a walk</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>walkItems-puddle.mp3</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Sølepytt</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Puddle</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Naming it happily, one word</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr"/>
+      <c r="J51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr"/>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Go for a walk</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>walkItems-stone.mp3</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Stein</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Stone</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Naming it happily, one word</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr"/>
+      <c r="J52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr"/>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Go for a walk</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>walkItems-bike.mp3</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Sykkel</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Bike</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Naming it happily, one word</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr"/>
+      <c r="J53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr"/>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Go for a walk</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>walkItems-squirrel.mp3</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Ekorn</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Squirrel</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Naming it happily, one word</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr"/>
+      <c r="J54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Walking song</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>walkSongSay.mp3</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Hør, jeg har laget en sang om turen vår!</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Listen, I've made a song about our walk!</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Proud, can not wait to share</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Help Mommy</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>foodSay.mp3</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Skal vi hjelpe mamma å lage mat? Velg hva dere skal lage!</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Shall we help Mommy make dinner? Choose what you're making!</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Hungry and helpful</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Help Mommy</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>dishSay.mp3</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Her er jobbene dine. Trykk når du er ferdig!</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Here are your jobs. Tap when you're done!</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Encouraging</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr"/>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Monki</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Goodnight</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>nightSay.mp3</t>
         </is>
       </c>
-      <c r="F44" s="3" t="inlineStr">
+      <c r="F58" s="3" t="inlineStr">
         <is>
           <t>Jeg er så trøtt nå. Takk for i dag! Nå kan dere leke sammen uten skjerm. Vi ses i morgen!</t>
         </is>
       </c>
-      <c r="G44" s="3" t="inlineStr">
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>I'm so sleepy now. Thank you for today! Now you can play together without a screen. See you tomorrow!</t>
         </is>
       </c>
-      <c r="H44" s="3" t="inlineStr">
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>Sleepy, yawning, warm</t>
         </is>
       </c>
-      <c r="I44" s="3" t="inlineStr"/>
-      <c r="J44" s="3" t="inlineStr"/>
+      <c r="I58" s="3" t="inlineStr"/>
+      <c r="J58" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J44"/>
+  <autoFilter ref="A1:J58"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:J44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:J58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>